<commit_message>
Lab 5 review fixes: price factor scales overage rate, wider forecast sheet headers
</commit_message>
<xml_diff>
--- a/lab5/out/lab5_recalculated.xlsx
+++ b/lab5/out/lab5_recalculated.xlsx
@@ -1181,7 +1181,7 @@
     <t xml:space="preserve">CAC payback, міс.</t>
   </si>
   <si>
-    <t xml:space="preserve">Припущення для ціни: COGS на акаунт 34,83 EUR і overage 467,5 EUR незмінні; змінюються базовий платіж і ціна будівлі; інші змінні витрати 6% від нової ARPA.</t>
+    <t xml:space="preserve">Припущення для ціни: змінюються всі ціни прайсу (базовий платіж, ціна будівлі, ставка overage 55 EUR); COGS на акаунт 34,83 EUR незмінний; інші змінні витрати 6% від нової ARPA.</t>
   </si>
   <si>
     <t xml:space="preserve">Припущення для CAC: 7 нових клієнтів сталі, тому CAC змінюється разом з acquisition spend.</t>
@@ -2016,11 +2016,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="29958937"/>
-        <c:axId val="79005867"/>
+        <c:axId val="34517882"/>
+        <c:axId val="69948636"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="29958937"/>
+        <c:axId val="34517882"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2086,7 +2086,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79005867"/>
+        <c:crossAx val="69948636"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2094,7 +2094,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="79005867"/>
+        <c:axId val="69948636"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2170,7 +2170,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29958937"/>
+        <c:crossAx val="34517882"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2231,14 +2231,14 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>126720</xdr:rowOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>78120</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
       <xdr:colOff>699840</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>148680</xdr:rowOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>100440</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -4259,14 +4259,14 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="13" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="0" width="12.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>303</v>
       </c>
@@ -5596,16 +5596,16 @@
         <v>355</v>
       </c>
       <c r="B11" s="12" t="n">
-        <f aca="false">(x5_rev_bu*B$2+x5_over)/x5_clients</f>
-        <v>186.95</v>
+        <f aca="false">(x5_rev_bu+x5_over)*B$2/x5_clients</f>
+        <v>185.08</v>
       </c>
       <c r="C11" s="12" t="n">
-        <f aca="false">(x5_rev_bu*C$2+x5_over)/x5_clients</f>
+        <f aca="false">(x5_rev_bu+x5_over)*C$2/x5_clients</f>
         <v>231.35</v>
       </c>
       <c r="D11" s="12" t="n">
-        <f aca="false">(x5_rev_bu*D$2+x5_over)/x5_clients</f>
-        <v>275.75</v>
+        <f aca="false">(x5_rev_bu+x5_over)*D$2/x5_clients</f>
+        <v>277.62</v>
       </c>
       <c r="E11" s="2"/>
     </row>
@@ -5615,7 +5615,7 @@
       </c>
       <c r="B12" s="7" t="n">
         <f aca="false">(B11-x5_cogs_pa)/B11</f>
-        <v>0.8136956405456</v>
+        <v>0.811813269937324</v>
       </c>
       <c r="C12" s="7" t="n">
         <f aca="false">(C11-x5_cogs_pa)/C11</f>
@@ -5623,7 +5623,7 @@
       </c>
       <c r="D12" s="7" t="n">
         <f aca="false">(D11-x5_cogs_pa)/D11</f>
-        <v>0.87369138712602</v>
+        <v>0.874542179958216</v>
       </c>
       <c r="E12" s="2"/>
     </row>
@@ -5633,7 +5633,7 @@
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">B11*(1-x5_ovshare)-x5_cogs_pa</f>
-        <v>140.9034</v>
+        <v>139.1456</v>
       </c>
       <c r="C13" s="12" t="n">
         <f aca="false">C11*(1-x5_ovshare)-x5_cogs_pa</f>
@@ -5641,7 +5641,7 @@
       </c>
       <c r="D13" s="12" t="n">
         <f aca="false">D11*(1-x5_ovshare)-x5_cogs_pa</f>
-        <v>224.3754</v>
+        <v>226.1332</v>
       </c>
       <c r="E13" s="2"/>
     </row>
@@ -5651,7 +5651,7 @@
       </c>
       <c r="B14" s="12" t="n">
         <f aca="false">B11*B12/x5_churn</f>
-        <v>5070.68</v>
+        <v>5008.34666666667</v>
       </c>
       <c r="C14" s="12" t="n">
         <f aca="false">C11*C12/x5_churn</f>
@@ -5659,7 +5659,7 @@
       </c>
       <c r="D14" s="12" t="n">
         <f aca="false">D11*D12/x5_churn</f>
-        <v>8030.68</v>
+        <v>8093.01333333333</v>
       </c>
       <c r="E14" s="2"/>
     </row>
@@ -5669,7 +5669,7 @@
       </c>
       <c r="B15" s="13" t="n">
         <f aca="false">B14/x5_cac</f>
-        <v>10.4396352941176</v>
+        <v>10.3113019607843</v>
       </c>
       <c r="C15" s="13" t="n">
         <f aca="false">C14/x5_cac</f>
@@ -5677,7 +5677,7 @@
       </c>
       <c r="D15" s="13" t="n">
         <f aca="false">D14/x5_cac</f>
-        <v>16.5337529411765</v>
+        <v>16.6620862745098</v>
       </c>
       <c r="E15" s="2"/>
     </row>
@@ -5687,7 +5687,7 @@
       </c>
       <c r="B16" s="13" t="n">
         <f aca="false">x5_fixed/B13</f>
-        <v>63.873547409076</v>
+        <v>64.6804498309684</v>
       </c>
       <c r="C16" s="13" t="n">
         <f aca="false">x5_fixed/C13</f>
@@ -5695,7 +5695,7 @@
       </c>
       <c r="D16" s="13" t="n">
         <f aca="false">x5_fixed/D13</f>
-        <v>40.1113491051158</v>
+        <v>39.7995517686036</v>
       </c>
       <c r="E16" s="2"/>
     </row>
@@ -5705,7 +5705,7 @@
       </c>
       <c r="B17" s="13" t="n">
         <f aca="false">(x5_fixed+x5_spend)/B13</f>
-        <v>88.0035542080603</v>
+        <v>89.1152864337787</v>
       </c>
       <c r="C17" s="13" t="n">
         <f aca="false">(x5_fixed+x5_spend)/C13</f>
@@ -5713,7 +5713,7 @@
       </c>
       <c r="D17" s="13" t="n">
         <f aca="false">(x5_fixed+x5_spend)/D13</f>
-        <v>55.2645254337151</v>
+        <v>54.8349379922983</v>
       </c>
       <c r="E17" s="2"/>
     </row>

</xml_diff>

<commit_message>
Lab 5 review fixes: single safety margin definition, x5_rev as formula, sensitivity labels inside bars, report details moved to appendix
</commit_message>
<xml_diff>
--- a/lab5/out/lab5_recalculated.xlsx
+++ b/lab5/out/lab5_recalculated.xlsx
@@ -25,6 +25,7 @@
     <definedName function="false" hidden="false" name="x5_be_cm" vbProcedure="false">'Break-even'!$D$2</definedName>
     <definedName function="false" hidden="false" name="x5_be_fixed" vbProcedure="false">'Break-even'!$D$3</definedName>
     <definedName function="false" hidden="false" name="x5_be_mos" vbProcedure="false">'Break-even'!$D$13</definedName>
+    <definedName function="false" hidden="false" name="x5_be_mos_o" vbProcedure="false">'Break-even'!$D$14</definedName>
     <definedName function="false" hidden="false" name="x5_be_o" vbProcedure="false">'Break-even'!$D$7</definedName>
     <definedName function="false" hidden="false" name="x5_be_o_b" vbProcedure="false">'Break-even'!$D$12</definedName>
     <definedName function="false" hidden="false" name="x5_be_o_int" vbProcedure="false">'Break-even'!$D$8</definedName>
@@ -33,7 +34,7 @@
     <definedName function="false" hidden="false" name="x5_be_p_b" vbProcedure="false">'Break-even'!$D$11</definedName>
     <definedName function="false" hidden="false" name="x5_be_p_int" vbProcedure="false">'Break-even'!$D$6</definedName>
     <definedName function="false" hidden="false" name="x5_be_p_rev" vbProcedure="false">'Break-even'!$D$9</definedName>
-    <definedName function="false" hidden="false" name="x5_be_steady" vbProcedure="false">'Break-even'!$D$14</definedName>
+    <definedName function="false" hidden="false" name="x5_be_steady" vbProcedure="false">'Break-even'!$D$15</definedName>
     <definedName function="false" hidden="false" name="x5_cac" vbProcedure="false">'Unit economics'!$D$2</definedName>
     <definedName function="false" hidden="false" name="x5_cap" vbProcedure="false">'Параметри ЛР5'!$C$25</definedName>
     <definedName function="false" hidden="false" name="x5_check" vbProcedure="false">'Параметри ЛР5'!$C$20</definedName>
@@ -93,7 +94,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="367">
   <si>
     <t xml:space="preserve">Ім'я</t>
   </si>
@@ -170,7 +171,10 @@
     <t xml:space="preserve">Revenue базового місяця Y3</t>
   </si>
   <si>
-    <t xml:space="preserve">ЛР № 4, сценарій 100%</t>
+    <t xml:space="preserve">Р</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ЛР № 4, сценарій 100%: сума двох рядків нижче</t>
   </si>
   <si>
     <t xml:space="preserve">x5_rev_bu</t>
@@ -374,9 +378,6 @@
     <t xml:space="preserve">Змінні витрати поза COGS, частка</t>
   </si>
   <si>
-    <t xml:space="preserve">Р</t>
-  </si>
-  <si>
     <t xml:space="preserve">x5_dm</t>
   </si>
   <si>
@@ -974,10 +975,19 @@
     <t xml:space="preserve">x5_be_mos</t>
   </si>
   <si>
-    <t xml:space="preserve">Запас Y3 ЛР № 4 над product BE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(50 − BE) / 50</t>
+    <t xml:space="preserve">Запас безпеки Y3 ЛР № 4 над product BE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(клієнти Y3 − BE) / клієнти Y3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x5_be_mos_o</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Запас безпеки M12 над operating BE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(клієнти M12 − BE) / клієнти M12</t>
   </si>
   <si>
     <t xml:space="preserve">x5_be_steady</t>
@@ -1355,6 +1365,10 @@
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="168" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1376,10 +1390,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="171" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2016,11 +2026,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="34517882"/>
-        <c:axId val="69948636"/>
+        <c:axId val="7697965"/>
+        <c:axId val="5784524"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="34517882"/>
+        <c:axId val="7697965"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2086,7 +2096,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69948636"/>
+        <c:crossAx val="5784524"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2094,7 +2104,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="69948636"/>
+        <c:axId val="5784524"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2170,7 +2180,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="34517882"/>
+        <c:crossAx val="7697965"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2571,32 +2581,33 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="6" t="n">
+        <f aca="false">x5_rev_bu+x5_over</f>
         <v>11567.5</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>11100</v>
@@ -2608,15 +2619,15 @@
         <v>9</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>467.5</v>
@@ -2628,15 +2639,15 @@
         <v>9</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C10" s="3" t="n">
         <v>1741.48</v>
@@ -2648,95 +2659,95 @@
         <v>9</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="C11" s="7" t="n">
         <v>50</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="C12" s="7" t="n">
         <v>1.7</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C13" s="3" t="n">
         <v>16</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C14" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="C14" s="7" t="n">
         <v>12</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C15" s="5" t="n">
         <v>0.1</v>
@@ -2748,35 +2759,35 @@
         <v>9</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C16" s="4" t="n">
         <v>70</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C17" s="5" t="n">
         <v>0.3</v>
@@ -2785,78 +2796,78 @@
         <v>16</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C18" s="4" t="n">
         <v>14</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C19" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="C19" s="7" t="n">
         <v>3</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C20" s="6" t="n">
+        <v>71</v>
+      </c>
+      <c r="C20" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>1200</v>
@@ -2865,18 +2876,18 @@
         <v>8</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C22" s="5" t="n">
         <v>0.015</v>
@@ -2885,18 +2896,18 @@
         <v>16</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C23" s="5" t="n">
         <v>0.01</v>
@@ -2905,18 +2916,18 @@
         <v>16</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C24" s="5" t="n">
         <v>0.035</v>
@@ -2925,58 +2936,58 @@
         <v>16</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C25" s="6" t="n">
+        <v>84</v>
+      </c>
+      <c r="C25" s="7" t="n">
         <v>36</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C26" s="6" t="n">
+        <v>87</v>
+      </c>
+      <c r="C26" s="7" t="n">
         <v>12</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C27" s="5" t="n">
         <v>0.2</v>
@@ -2988,7 +2999,7 @@
         <v>9</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3001,12 +3012,12 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="C29" s="7" t="n">
+        <v>93</v>
+      </c>
+      <c r="C29" s="8" t="n">
         <f aca="false">x5_pay+x5_bad+x5_partner</f>
         <v>0.06</v>
       </c>
@@ -3014,10 +3025,10 @@
         <v>16</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3027,7 +3038,7 @@
       <c r="B30" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C30" s="8" t="n">
+      <c r="C30" s="9" t="n">
         <f aca="false">(1+x5_disc)^(1/12)-1</f>
         <v>0.00797414042890376</v>
       </c>
@@ -3035,7 +3046,7 @@
         <v>16</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>96</v>
@@ -3086,7 +3097,7 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>100</v>
@@ -3120,7 +3131,7 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>109</v>
@@ -3137,7 +3148,7 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>113</v>
@@ -3154,7 +3165,7 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>117</v>
@@ -3214,7 +3225,7 @@
         <v>133</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>134</v>
@@ -3304,11 +3315,11 @@
       <c r="B2" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="C2" s="9" t="n">
+      <c r="C2" s="10" t="n">
         <f aca="false">x5_leads</f>
         <v>70</v>
       </c>
-      <c r="D2" s="10"/>
+      <c r="D2" s="11"/>
       <c r="E2" s="2" t="s">
         <v>152</v>
       </c>
@@ -3320,11 +3331,11 @@
       <c r="B3" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="C3" s="9" t="n">
+      <c r="C3" s="10" t="n">
         <f aca="false">C2*x5_act</f>
         <v>21</v>
       </c>
-      <c r="D3" s="11" t="n">
+      <c r="D3" s="12" t="n">
         <f aca="false">C3/C2</f>
         <v>0.3</v>
       </c>
@@ -3339,11 +3350,11 @@
       <c r="B4" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="C4" s="9" t="n">
+      <c r="C4" s="10" t="n">
         <f aca="false">x5_kept</f>
         <v>14</v>
       </c>
-      <c r="D4" s="11" t="n">
+      <c r="D4" s="12" t="n">
         <f aca="false">C4/C3</f>
         <v>0.666666666666667</v>
       </c>
@@ -3358,11 +3369,11 @@
       <c r="B5" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="10" t="n">
         <f aca="false">x5_new</f>
         <v>7</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="12" t="n">
         <f aca="false">C5/C4</f>
         <v>0.5</v>
       </c>
@@ -3388,7 +3399,7 @@
       <c r="B8" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="C8" s="11" t="n">
+      <c r="C8" s="12" t="n">
         <f aca="false">C5/C2</f>
         <v>0.1</v>
       </c>
@@ -3400,7 +3411,7 @@
       <c r="B9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="C9" s="11" t="n">
+      <c r="C9" s="12" t="n">
         <f aca="false">C5/C3</f>
         <v>0.333333333333333</v>
       </c>
@@ -3412,7 +3423,7 @@
       <c r="B10" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="10" t="n">
         <f aca="false">C3*x5_check+C4*(x5_pilot_m-x5_check)</f>
         <v>49</v>
       </c>
@@ -3424,7 +3435,7 @@
       <c r="B11" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="6" t="n">
         <f aca="false">C10*x5_cogs_unit</f>
         <v>784</v>
       </c>
@@ -3434,9 +3445,9 @@
         <v>171</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C12" s="12" t="n">
+        <v>74</v>
+      </c>
+      <c r="C12" s="6" t="n">
         <f aca="false">x5_events</f>
         <v>1200</v>
       </c>
@@ -3448,7 +3459,7 @@
       <c r="B13" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="6" t="n">
         <f aca="false">x5_spend-C11-C12</f>
         <v>1416</v>
       </c>
@@ -3460,7 +3471,7 @@
       <c r="B14" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="6" t="n">
         <f aca="false">C11+C12+C13</f>
         <v>3400</v>
       </c>
@@ -3472,7 +3483,7 @@
       <c r="B15" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="C15" s="12" t="n">
+      <c r="C15" s="6" t="n">
         <f aca="false">x5_spend/C2</f>
         <v>48.5714285714286</v>
       </c>
@@ -3484,7 +3495,7 @@
       <c r="B16" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C16" s="12" t="n">
+      <c r="C16" s="6" t="n">
         <f aca="false">x5_spend/C3</f>
         <v>161.904761904762</v>
       </c>
@@ -3542,7 +3553,7 @@
       <c r="C2" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="D2" s="12" t="n">
+      <c r="D2" s="6" t="n">
         <f aca="false">x5_spend/x5_new</f>
         <v>485.714285714286</v>
       </c>
@@ -3560,7 +3571,7 @@
       <c r="C3" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="D3" s="12" t="n">
+      <c r="D3" s="6" t="n">
         <f aca="false">x5_rev/x5_clients</f>
         <v>231.35</v>
       </c>
@@ -3578,7 +3589,7 @@
       <c r="C4" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="D4" s="12" t="n">
+      <c r="D4" s="6" t="n">
         <f aca="false">x5_rev/x5_scale</f>
         <v>136.088235294118</v>
       </c>
@@ -3596,7 +3607,7 @@
       <c r="C5" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="6" t="n">
         <f aca="false">x5_cogs/x5_clients</f>
         <v>34.8296</v>
       </c>
@@ -3614,7 +3625,7 @@
       <c r="C6" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="6" t="n">
         <f aca="false">x5_arpa-x5_cogs_pa</f>
         <v>196.5204</v>
       </c>
@@ -3632,7 +3643,7 @@
       <c r="C7" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="8" t="n">
         <f aca="false">(x5_rev-x5_cogs)/x5_rev</f>
         <v>0.84945061594986</v>
       </c>
@@ -3650,7 +3661,7 @@
       <c r="C8" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="6" t="n">
         <f aca="false">x5_arpa*x5_ovshare</f>
         <v>13.881</v>
       </c>
@@ -3668,7 +3679,7 @@
       <c r="C9" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="6" t="n">
         <f aca="false">x5_arpa-x5_cogs_pa-x5_ov</f>
         <v>182.6394</v>
       </c>
@@ -3686,7 +3697,7 @@
       <c r="C10" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="8" t="n">
         <f aca="false">x5_cm/x5_arpa</f>
         <v>0.78945061594986</v>
       </c>
@@ -3709,7 +3720,7 @@
         <v>1.5</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3722,7 +3733,7 @@
       <c r="C12" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="6" t="n">
         <f aca="false">x5_churn*x5_rev</f>
         <v>347.025</v>
       </c>
@@ -3740,7 +3751,7 @@
       <c r="C13" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="6" t="n">
         <f aca="false">x5_over/x5_episode</f>
         <v>38.9583333333333</v>
       </c>
@@ -3758,7 +3769,7 @@
       <c r="C14" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="6" t="n">
         <f aca="false">x5_contr</f>
         <v>38.9583333333333</v>
       </c>
@@ -3812,7 +3823,7 @@
       <c r="C17" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="D17" s="6" t="n">
         <f aca="false">x5_arpa*x5_gm/x5_churn</f>
         <v>6550.68</v>
       </c>
@@ -3853,7 +3864,7 @@
         <v>2.47157183536308</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3871,7 +3882,7 @@
         <v>33.3333333333333</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3884,7 +3895,7 @@
       <c r="C21" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="D21" s="12" t="n">
+      <c r="D21" s="6" t="n">
         <f aca="false">x5_cm/x5_churn</f>
         <v>6087.98</v>
       </c>
@@ -3902,7 +3913,7 @@
       <c r="C22" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="D22" s="12" t="n">
+      <c r="D22" s="6" t="n">
         <f aca="false">x5_gp/x5_grc</f>
         <v>5889.50229370871</v>
       </c>
@@ -3920,7 +3931,7 @@
       <c r="C23" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D23" s="12" t="n">
+      <c r="D23" s="6" t="n">
         <f aca="false">x5_gp*(1+x5_dm)/(x5_churn+x5_dm)</f>
         <v>5216.37827820248</v>
       </c>
@@ -3938,7 +3949,7 @@
       <c r="C24" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="D24" s="12" t="n">
+      <c r="D24" s="6" t="n">
         <f aca="false">x5_gp*(1-(1-x5_churn)^x5_cap)/x5_churn</f>
         <v>4362.57167590805</v>
       </c>
@@ -3961,7 +3972,7 @@
         <v>2.6594167836419</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -3980,7 +3991,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -4013,7 +4024,7 @@
       <c r="C2" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="D2" s="12" t="n">
+      <c r="D2" s="6" t="n">
         <f aca="false">x5_cm</f>
         <v>182.6394</v>
       </c>
@@ -4028,7 +4039,7 @@
       <c r="C3" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="D3" s="12" t="n">
+      <c r="D3" s="6" t="n">
         <f aca="false">x5_fixed</f>
         <v>9000</v>
       </c>
@@ -4043,7 +4054,7 @@
       <c r="C4" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="D4" s="12" t="n">
+      <c r="D4" s="6" t="n">
         <f aca="false">x5_spend</f>
         <v>3400</v>
       </c>
@@ -4073,7 +4084,7 @@
       <c r="C6" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="10" t="n">
         <f aca="false">ROUNDUP(x5_be_p-0.000000001,0)</f>
         <v>50</v>
       </c>
@@ -4103,7 +4114,7 @@
       <c r="C8" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="10" t="n">
         <f aca="false">ROUNDUP(x5_be_o-0.000000001,0)</f>
         <v>68</v>
       </c>
@@ -4118,7 +4129,7 @@
       <c r="C9" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="6" t="n">
         <f aca="false">x5_be_fixed/x5_cmr</f>
         <v>11400.3331154176</v>
       </c>
@@ -4133,7 +4144,7 @@
       <c r="C10" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="6" t="n">
         <f aca="false">(x5_be_fixed+x5_be_acq)/x5_cmr</f>
         <v>15707.1256256865</v>
       </c>
@@ -4178,7 +4189,7 @@
       <c r="C13" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="8" t="n">
         <f aca="false">(x5_clients-x5_be_p)/x5_clients</f>
         <v>0.0144514272385915</v>
       </c>
@@ -4193,9 +4204,9 @@
       <c r="C14" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="D14" s="13" t="n">
-        <f aca="false">x5_new/x5_churn</f>
-        <v>233.333333333333</v>
+      <c r="D14" s="8" t="n">
+        <f aca="false">('Прогноз 12 міс.'!$F$13-x5_be_o)/'Прогноз 12 міс.'!$F$13</f>
+        <v>0.0496024063526117</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4208,9 +4219,9 @@
       <c r="C15" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="D15" s="9" t="n">
-        <f aca="false">'Прогноз 12 міс.'!$F$16</f>
-        <v>8</v>
+      <c r="D15" s="13" t="n">
+        <f aca="false">x5_new/x5_churn</f>
+        <v>233.333333333333</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4221,9 +4232,24 @@
         <v>302</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="D16" s="9" t="n">
+        <v>303</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <f aca="false">'Прогноз 12 міс.'!$F$16</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="D17" s="10" t="n">
         <f aca="false">'Прогноз 12 міс.'!$F$17</f>
         <v>12</v>
       </c>
@@ -4268,64 +4294,64 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>159</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4333,7 +4359,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C2" s="13" t="n">
         <f aca="false">0</f>
@@ -4413,7 +4439,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="C3" s="13" t="n">
         <f aca="false">F2</f>
@@ -4493,7 +4519,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C4" s="13" t="n">
         <f aca="false">F3</f>
@@ -4573,7 +4599,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="C5" s="13" t="n">
         <f aca="false">F4</f>
@@ -4653,7 +4679,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="C6" s="13" t="n">
         <f aca="false">F5</f>
@@ -4733,7 +4759,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="C7" s="13" t="n">
         <f aca="false">F6</f>
@@ -4813,7 +4839,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="C8" s="13" t="n">
         <f aca="false">F7</f>
@@ -4893,7 +4919,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="C9" s="13" t="n">
         <f aca="false">F8</f>
@@ -4973,7 +4999,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="C10" s="13" t="n">
         <f aca="false">F9</f>
@@ -5053,7 +5079,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="C11" s="13" t="n">
         <f aca="false">F10</f>
@@ -5133,7 +5159,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="C12" s="13" t="n">
         <f aca="false">F11</f>
@@ -5213,7 +5239,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="C13" s="13" t="n">
         <f aca="false">F12</f>
@@ -5290,7 +5316,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -5302,7 +5328,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -5315,7 +5341,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -5328,7 +5354,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -5341,7 +5367,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -5354,7 +5380,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -5367,7 +5393,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -5379,7 +5405,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -5427,24 +5453,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="B2" s="23" t="n">
         <f aca="false">1-x5_delta</f>
@@ -5458,33 +5484,33 @@
         <v>1.2</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="24" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="7" t="n">
+      <c r="B4" s="8" t="n">
         <f aca="false">x5_churn*B$2</f>
         <v>0.024</v>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="8" t="n">
         <f aca="false">x5_churn*C$2</f>
         <v>0.03</v>
       </c>
-      <c r="D4" s="7" t="n">
+      <c r="D4" s="8" t="n">
         <f aca="false">x5_churn*D$2</f>
         <v>0.036</v>
       </c>
@@ -5492,17 +5518,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>349</v>
-      </c>
-      <c r="B5" s="12" t="n">
+        <v>352</v>
+      </c>
+      <c r="B5" s="6" t="n">
         <f aca="false">x5_arpa*x5_gm/B4</f>
         <v>8188.35</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="6" t="n">
         <f aca="false">x5_arpa*x5_gm/C4</f>
         <v>6550.68</v>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="6" t="n">
         <f aca="false">x5_arpa*x5_gm/D4</f>
         <v>5458.9</v>
       </c>
@@ -5528,7 +5554,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="B7" s="13" t="n">
         <f aca="false">x5_new/B4</f>
@@ -5546,17 +5572,17 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>351</v>
-      </c>
-      <c r="B8" s="9" t="n">
+        <v>354</v>
+      </c>
+      <c r="B8" s="10" t="n">
         <f aca="false">IF(x5_be_p&gt;=x5_new/B4,"не досягнуто",IF(ROUNDUP(LN(1-x5_be_p*B4/x5_new)/LN(1-B4)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-x5_be_p*B4/x5_new)/LN(1-B4)-0.000000001,0)))</f>
         <v>8</v>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="10" t="n">
         <f aca="false">IF(x5_be_p&gt;=x5_new/C4,"не досягнуто",IF(ROUNDUP(LN(1-x5_be_p*C4/x5_new)/LN(1-C4)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-x5_be_p*C4/x5_new)/LN(1-C4)-0.000000001,0)))</f>
         <v>8</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="10" t="n">
         <f aca="false">IF(x5_be_p&gt;=x5_new/D4,"не досягнуто",IF(ROUNDUP(LN(1-x5_be_p*D4/x5_new)/LN(1-D4)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-x5_be_p*D4/x5_new)/LN(1-D4)-0.000000001,0)))</f>
         <v>8</v>
       </c>
@@ -5564,17 +5590,17 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="B9" s="9" t="n">
+        <v>355</v>
+      </c>
+      <c r="B9" s="10" t="n">
         <f aca="false">IF(x5_be_o&gt;=x5_new/B4,"не досягнуто",IF(ROUNDUP(LN(1-x5_be_o*B4/x5_new)/LN(1-B4)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-x5_be_o*B4/x5_new)/LN(1-B4)-0.000000001,0)))</f>
         <v>11</v>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="10" t="n">
         <f aca="false">IF(x5_be_o&gt;=x5_new/C4,"не досягнуто",IF(ROUNDUP(LN(1-x5_be_o*C4/x5_new)/LN(1-C4)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-x5_be_o*C4/x5_new)/LN(1-C4)-0.000000001,0)))</f>
         <v>12</v>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="10" t="n">
         <f aca="false">IF(x5_be_o&gt;=x5_new/D4,"не досягнуто",IF(ROUNDUP(LN(1-x5_be_o*D4/x5_new)/LN(1-D4)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-x5_be_o*D4/x5_new)/LN(1-D4)-0.000000001,0)))</f>
         <v>12</v>
       </c>
@@ -5582,28 +5608,28 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="24" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>355</v>
-      </c>
-      <c r="B11" s="12" t="n">
+        <v>358</v>
+      </c>
+      <c r="B11" s="6" t="n">
         <f aca="false">(x5_rev_bu+x5_over)*B$2/x5_clients</f>
         <v>185.08</v>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="6" t="n">
         <f aca="false">(x5_rev_bu+x5_over)*C$2/x5_clients</f>
         <v>231.35</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="6" t="n">
         <f aca="false">(x5_rev_bu+x5_over)*D$2/x5_clients</f>
         <v>277.62</v>
       </c>
@@ -5613,15 +5639,15 @@
       <c r="A12" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B12" s="8" t="n">
         <f aca="false">(B11-x5_cogs_pa)/B11</f>
         <v>0.811813269937324</v>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="8" t="n">
         <f aca="false">(C11-x5_cogs_pa)/C11</f>
         <v>0.84945061594986</v>
       </c>
-      <c r="D12" s="7" t="n">
+      <c r="D12" s="8" t="n">
         <f aca="false">(D11-x5_cogs_pa)/D11</f>
         <v>0.874542179958216</v>
       </c>
@@ -5629,17 +5655,17 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="B13" s="12" t="n">
+        <v>359</v>
+      </c>
+      <c r="B13" s="6" t="n">
         <f aca="false">B11*(1-x5_ovshare)-x5_cogs_pa</f>
         <v>139.1456</v>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="6" t="n">
         <f aca="false">C11*(1-x5_ovshare)-x5_cogs_pa</f>
         <v>182.6394</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="6" t="n">
         <f aca="false">D11*(1-x5_ovshare)-x5_cogs_pa</f>
         <v>226.1332</v>
       </c>
@@ -5647,17 +5673,17 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>349</v>
-      </c>
-      <c r="B14" s="12" t="n">
+        <v>352</v>
+      </c>
+      <c r="B14" s="6" t="n">
         <f aca="false">B11*B12/x5_churn</f>
         <v>5008.34666666667</v>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="6" t="n">
         <f aca="false">C11*C12/x5_churn</f>
         <v>6550.68</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="6" t="n">
         <f aca="false">D11*D12/x5_churn</f>
         <v>8093.01333333333</v>
       </c>
@@ -5683,7 +5709,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B16" s="13" t="n">
         <f aca="false">x5_fixed/B13</f>
@@ -5701,7 +5727,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="B17" s="13" t="n">
         <f aca="false">(x5_fixed+x5_spend)/B13</f>
@@ -5719,17 +5745,17 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>351</v>
-      </c>
-      <c r="B18" s="9" t="n">
+        <v>354</v>
+      </c>
+      <c r="B18" s="10" t="n">
         <f aca="false">IF(B16&gt;=x5_new/x5_churn,"не досягнуто",IF(ROUNDUP(LN(1-B16*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-B16*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)))</f>
         <v>11</v>
       </c>
-      <c r="C18" s="9" t="n">
+      <c r="C18" s="10" t="n">
         <f aca="false">IF(C16&gt;=x5_new/x5_churn,"не досягнуто",IF(ROUNDUP(LN(1-C16*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-C16*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)))</f>
         <v>8</v>
       </c>
-      <c r="D18" s="9" t="n">
+      <c r="D18" s="10" t="n">
         <f aca="false">IF(D16&gt;=x5_new/x5_churn,"не досягнуто",IF(ROUNDUP(LN(1-D16*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-D16*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)))</f>
         <v>7</v>
       </c>
@@ -5737,17 +5763,17 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="B19" s="9" t="str">
+        <v>355</v>
+      </c>
+      <c r="B19" s="10" t="str">
         <f aca="false">IF(B17&gt;=x5_new/x5_churn,"не досягнуто",IF(ROUNDUP(LN(1-B17*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-B17*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)))</f>
         <v>не досягнуто</v>
       </c>
-      <c r="C19" s="9" t="n">
+      <c r="C19" s="10" t="n">
         <f aca="false">IF(C17&gt;=x5_new/x5_churn,"не досягнуто",IF(ROUNDUP(LN(1-C17*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-C17*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)))</f>
         <v>12</v>
       </c>
-      <c r="D19" s="9" t="n">
+      <c r="D19" s="10" t="n">
         <f aca="false">IF(D17&gt;=x5_new/x5_churn,"не досягнуто",IF(ROUNDUP(LN(1-D17*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-D17*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)))</f>
         <v>9</v>
       </c>
@@ -5761,22 +5787,22 @@
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="B21" s="12" t="n">
+      <c r="B21" s="6" t="n">
         <f aca="false">x5_spend*B$2</f>
         <v>2720</v>
       </c>
-      <c r="C21" s="12" t="n">
+      <c r="C21" s="6" t="n">
         <f aca="false">x5_spend*C$2</f>
         <v>3400</v>
       </c>
-      <c r="D21" s="12" t="n">
+      <c r="D21" s="6" t="n">
         <f aca="false">x5_spend*D$2</f>
         <v>4080</v>
       </c>
@@ -5784,17 +5810,17 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="B22" s="12" t="n">
+        <v>363</v>
+      </c>
+      <c r="B22" s="6" t="n">
         <f aca="false">B21/x5_new</f>
         <v>388.571428571429</v>
       </c>
-      <c r="C22" s="12" t="n">
+      <c r="C22" s="6" t="n">
         <f aca="false">C21/x5_new</f>
         <v>485.714285714286</v>
       </c>
-      <c r="D22" s="12" t="n">
+      <c r="D22" s="6" t="n">
         <f aca="false">D21/x5_new</f>
         <v>582.857142857143</v>
       </c>
@@ -5820,7 +5846,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="B24" s="13" t="n">
         <f aca="false">B22/x5_gp</f>
@@ -5838,7 +5864,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B25" s="13" t="n">
         <f aca="false">x5_fixed/x5_cm</f>
@@ -5856,7 +5882,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="B26" s="13" t="n">
         <f aca="false">(x5_fixed+B21)/x5_cm</f>
@@ -5874,17 +5900,17 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="B27" s="9" t="n">
+        <v>355</v>
+      </c>
+      <c r="B27" s="10" t="n">
         <f aca="false">IF(B26&gt;=x5_new/x5_churn,"не досягнуто",IF(ROUNDUP(LN(1-B26*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-B26*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)))</f>
         <v>11</v>
       </c>
-      <c r="C27" s="9" t="n">
+      <c r="C27" s="10" t="n">
         <f aca="false">IF(C26&gt;=x5_new/x5_churn,"не досягнуто",IF(ROUNDUP(LN(1-C26*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-C26*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)))</f>
         <v>12</v>
       </c>
-      <c r="D27" s="9" t="str">
+      <c r="D27" s="10" t="str">
         <f aca="false">IF(D26&gt;=x5_new/x5_churn,"не досягнуто",IF(ROUNDUP(LN(1-D26*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-D26*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)))</f>
         <v>не досягнуто</v>
       </c>
@@ -5892,12 +5918,12 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Lab 5 consistency: scale trigger of lab 3 fires in M8, cloud recalculated by buildings, fixed cost headroom, cash burn reconciliation with lab 3, CAC threshold 578 EUR, operating safety margin Y3 in workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lab5/out/lab5_recalculated.xlsx
+++ b/lab5/out/lab5_recalculated.xlsx
@@ -34,7 +34,7 @@
     <definedName function="false" hidden="false" name="x5_be_p_b" vbProcedure="false">'Break-even'!$D$11</definedName>
     <definedName function="false" hidden="false" name="x5_be_p_int" vbProcedure="false">'Break-even'!$D$6</definedName>
     <definedName function="false" hidden="false" name="x5_be_p_rev" vbProcedure="false">'Break-even'!$D$9</definedName>
-    <definedName function="false" hidden="false" name="x5_be_steady" vbProcedure="false">'Break-even'!$D$15</definedName>
+    <definedName function="false" hidden="false" name="x5_be_steady" vbProcedure="false">'Break-even'!$D$17</definedName>
     <definedName function="false" hidden="false" name="x5_cac" vbProcedure="false">'Unit economics'!$D$2</definedName>
     <definedName function="false" hidden="false" name="x5_cap" vbProcedure="false">'Параметри ЛР5'!$C$25</definedName>
     <definedName function="false" hidden="false" name="x5_check" vbProcedure="false">'Параметри ЛР5'!$C$20</definedName>
@@ -53,6 +53,7 @@
     <definedName function="false" hidden="false" name="x5_events" vbProcedure="false">'Параметри ЛР5'!$C$21</definedName>
     <definedName function="false" hidden="false" name="x5_exp" vbProcedure="false">'Unit economics'!$D$14</definedName>
     <definedName function="false" hidden="false" name="x5_fixed" vbProcedure="false">'Параметри ЛР5'!$C$5</definedName>
+    <definedName function="false" hidden="false" name="x5_fix_room" vbProcedure="false">'Break-even'!$D$16</definedName>
     <definedName function="false" hidden="false" name="x5_gm" vbProcedure="false">'Unit economics'!$D$7</definedName>
     <definedName function="false" hidden="false" name="x5_gp" vbProcedure="false">'Unit economics'!$D$6</definedName>
     <definedName function="false" hidden="false" name="x5_grc" vbProcedure="false">'Unit economics'!$D$15</definedName>
@@ -68,6 +69,7 @@
     <definedName function="false" hidden="false" name="x5_ltv_cm" vbProcedure="false">'Unit economics'!$D$21</definedName>
     <definedName function="false" hidden="false" name="x5_ltv_disc" vbProcedure="false">'Unit economics'!$D$23</definedName>
     <definedName function="false" hidden="false" name="x5_ltv_rev" vbProcedure="false">'Unit economics'!$D$22</definedName>
+    <definedName function="false" hidden="false" name="x5_mos_oy3" vbProcedure="false">'Break-even'!$D$15</definedName>
     <definedName function="false" hidden="false" name="x5_new" vbProcedure="false">'Параметри ЛР5'!$C$3</definedName>
     <definedName function="false" hidden="false" name="x5_nrc" vbProcedure="false">'Unit economics'!$D$16</definedName>
     <definedName function="false" hidden="false" name="x5_ov" vbProcedure="false">'Unit economics'!$D$8</definedName>
@@ -94,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="372">
   <si>
     <t xml:space="preserve">Ім'я</t>
   </si>
@@ -988,6 +990,21 @@
   </si>
   <si>
     <t xml:space="preserve">(клієнти M12 − BE) / клієнти M12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x5_mos_oy3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Запас безпеки Y3 ЛР № 4 над operating BE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x5_fix_room</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Допустимий приріст fixed OPEX для operating BE у M12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(клієнти M12 − operating BE) × CM, EUR на місяць</t>
   </si>
   <si>
     <t xml:space="preserve">x5_be_steady</t>
@@ -2026,11 +2043,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="7697965"/>
-        <c:axId val="5784524"/>
+        <c:axId val="78373576"/>
+        <c:axId val="50989611"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="7697965"/>
+        <c:axId val="78373576"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2096,7 +2113,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5784524"/>
+        <c:crossAx val="50989611"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2104,7 +2121,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="5784524"/>
+        <c:axId val="50989611"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2180,7 +2197,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7697965"/>
+        <c:crossAx val="78373576"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3991,7 +4008,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -4209,7 +4226,7 @@
         <v>0.0496024063526117</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
         <v>298</v>
       </c>
@@ -4217,39 +4234,69 @@
         <v>299</v>
       </c>
       <c r="C15" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <f aca="false">(x5_clients-x5_be_o)/x5_clients</f>
+        <v>-0.357866922471274</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="B16" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <f aca="false">('Прогноз 12 міс.'!$F$13-x5_be_o)*x5_be_cm</f>
+        <v>647.171081748955</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="D17" s="13" t="n">
         <f aca="false">x5_new/x5_churn</f>
         <v>233.333333333333</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
-        <v>301</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="D16" s="10" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="D18" s="10" t="n">
         <f aca="false">'Прогноз 12 міс.'!$F$16</f>
         <v>8</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="D17" s="10" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="D19" s="10" t="n">
         <f aca="false">'Прогноз 12 міс.'!$F$17</f>
         <v>12</v>
       </c>
@@ -4294,64 +4341,64 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>159</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4359,7 +4406,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="C2" s="13" t="n">
         <f aca="false">0</f>
@@ -4439,7 +4486,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="C3" s="13" t="n">
         <f aca="false">F2</f>
@@ -4519,7 +4566,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="C4" s="13" t="n">
         <f aca="false">F3</f>
@@ -4599,7 +4646,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="C5" s="13" t="n">
         <f aca="false">F4</f>
@@ -4679,7 +4726,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="C6" s="13" t="n">
         <f aca="false">F5</f>
@@ -4759,7 +4806,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="C7" s="13" t="n">
         <f aca="false">F6</f>
@@ -4839,7 +4886,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="C8" s="13" t="n">
         <f aca="false">F7</f>
@@ -4919,7 +4966,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="C9" s="13" t="n">
         <f aca="false">F8</f>
@@ -4999,7 +5046,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="C10" s="13" t="n">
         <f aca="false">F9</f>
@@ -5079,7 +5126,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="C11" s="13" t="n">
         <f aca="false">F10</f>
@@ -5159,7 +5206,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="C12" s="13" t="n">
         <f aca="false">F11</f>
@@ -5239,7 +5286,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="C13" s="13" t="n">
         <f aca="false">F12</f>
@@ -5316,7 +5363,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -5328,7 +5375,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -5341,7 +5388,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -5354,7 +5401,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -5367,7 +5414,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -5380,7 +5427,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -5393,7 +5440,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -5405,7 +5452,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -5453,24 +5500,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="B2" s="23" t="n">
         <f aca="false">1-x5_delta</f>
@@ -5484,18 +5531,18 @@
         <v>1.2</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="24" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5518,7 +5565,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="B5" s="6" t="n">
         <f aca="false">x5_arpa*x5_gm/B4</f>
@@ -5554,7 +5601,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="B7" s="13" t="n">
         <f aca="false">x5_new/B4</f>
@@ -5572,7 +5619,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="B8" s="10" t="n">
         <f aca="false">IF(x5_be_p&gt;=x5_new/B4,"не досягнуто",IF(ROUNDUP(LN(1-x5_be_p*B4/x5_new)/LN(1-B4)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-x5_be_p*B4/x5_new)/LN(1-B4)-0.000000001,0)))</f>
@@ -5590,7 +5637,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="B9" s="10" t="n">
         <f aca="false">IF(x5_be_o&gt;=x5_new/B4,"не досягнуто",IF(ROUNDUP(LN(1-x5_be_o*B4/x5_new)/LN(1-B4)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-x5_be_o*B4/x5_new)/LN(1-B4)-0.000000001,0)))</f>
@@ -5608,18 +5655,18 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="24" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="B11" s="6" t="n">
         <f aca="false">(x5_rev_bu+x5_over)*B$2/x5_clients</f>
@@ -5655,7 +5702,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">B11*(1-x5_ovshare)-x5_cogs_pa</f>
@@ -5673,7 +5720,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="B14" s="6" t="n">
         <f aca="false">B11*B12/x5_churn</f>
@@ -5709,7 +5756,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="B16" s="13" t="n">
         <f aca="false">x5_fixed/B13</f>
@@ -5727,7 +5774,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="B17" s="13" t="n">
         <f aca="false">(x5_fixed+x5_spend)/B13</f>
@@ -5745,7 +5792,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="B18" s="10" t="n">
         <f aca="false">IF(B16&gt;=x5_new/x5_churn,"не досягнуто",IF(ROUNDUP(LN(1-B16*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-B16*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)))</f>
@@ -5763,7 +5810,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="B19" s="10" t="str">
         <f aca="false">IF(B17&gt;=x5_new/x5_churn,"не досягнуто",IF(ROUNDUP(LN(1-B17*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-B17*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)))</f>
@@ -5787,7 +5834,7 @@
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5810,7 +5857,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="B22" s="6" t="n">
         <f aca="false">B21/x5_new</f>
@@ -5846,7 +5893,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="B24" s="13" t="n">
         <f aca="false">B22/x5_gp</f>
@@ -5864,7 +5911,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="B25" s="13" t="n">
         <f aca="false">x5_fixed/x5_cm</f>
@@ -5882,7 +5929,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="B26" s="13" t="n">
         <f aca="false">(x5_fixed+B21)/x5_cm</f>
@@ -5900,7 +5947,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="B27" s="10" t="n">
         <f aca="false">IF(B26&gt;=x5_new/x5_churn,"не досягнуто",IF(ROUNDUP(LN(1-B26*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)&gt;x5_h,"не досягнуто",ROUNDUP(LN(1-B26*x5_churn/x5_new)/LN(1-x5_churn)-0.000000001,0)))</f>
@@ -5918,12 +5965,12 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
     </row>
   </sheetData>

</xml_diff>